<commit_message>
Updated readme and updated the metadata files
</commit_message>
<xml_diff>
--- a/metadata/dominance_meta_corrected_outlier_corrected.xlsx
+++ b/metadata/dominance_meta_corrected_outlier_corrected.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/f8cb5b7fcd4c426a/Dokument/Master courses/MASTER THESIS/R project-Master Thesis/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="83" documentId="8_{E6DE9369-E5A4-41F0-AC43-5D1C5DBAA4C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D82E6ADB-3A11-4A24-871B-71215146246D}"/>
+  <xr:revisionPtr revIDLastSave="91" documentId="8_{E6DE9369-E5A4-41F0-AC43-5D1C5DBAA4C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{072B3E9C-09E0-49DB-9C7E-142293E9F969}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{FDDCB103-F9DC-4D01-9EF3-13268919B821}"/>
   </bookViews>
@@ -50,7 +50,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="946" uniqueCount="568">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="946" uniqueCount="569">
   <si>
     <t>Run</t>
   </si>
@@ -1621,9 +1621,6 @@
     <t>TF-2581-18_S15_L001_R2_001.fastq.gz</t>
   </si>
   <si>
-    <t>Possibly ambigous sex</t>
-  </si>
-  <si>
     <t>ERR12383278</t>
   </si>
   <si>
@@ -1723,9 +1720,6 @@
     <t>DD Homozygote</t>
   </si>
   <si>
-    <t>Most likely mislabel. Relabeled as female</t>
-  </si>
-  <si>
     <t>EE</t>
   </si>
   <si>
@@ -1754,6 +1748,15 @@
   </si>
   <si>
     <t xml:space="preserve">Had TF ID: TF2581-71, and Sample ID: 72 before. This change should be correct </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Possibly ambigous sex, below -50 in the PCA,strays from the other female samples.  But was kept in my thesis </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Possibly ambigous sex, below 50 in the PCA, strays from the other male samples.  But was kept in my thesis </t>
+  </si>
+  <si>
+    <t xml:space="preserve">NOTE! I relabeled from Male to Female here. Clustered deep with female samples in PCA. But was noted as Male during sampling/sequencing </t>
   </si>
 </sst>
 </file>
@@ -1979,7 +1982,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="7" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -2074,27 +2077,12 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="22">
-    <dxf>
-      <alignment vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top/>
-        <bottom/>
-      </border>
-    </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
       <alignment vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -2407,26 +2395,42 @@
       </border>
     </dxf>
     <dxf>
-      <border>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
         <bottom style="thin">
           <color indexed="64"/>
         </bottom>
       </border>
     </dxf>
     <dxf>
-      <border diagonalUp="0" diagonalDown="0">
+      <alignment vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <border>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
         <left style="thin">
           <color indexed="64"/>
         </left>
         <right style="thin">
           <color indexed="64"/>
         </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
+        <top/>
+        <bottom/>
       </border>
     </dxf>
   </dxfs>
@@ -2473,29 +2477,29 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{D4DDD6FC-9AB0-4E27-B100-332C5258E37E}" name="metadata_for_manual_correction3" displayName="metadata_for_manual_correction3" ref="A1:Q71" tableType="queryTable" totalsRowShown="0" headerRowDxfId="1" dataDxfId="0" headerRowBorderDxfId="20" tableBorderDxfId="21" totalsRowBorderDxfId="19">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{D4DDD6FC-9AB0-4E27-B100-332C5258E37E}" name="metadata_for_manual_correction3" displayName="metadata_for_manual_correction3" ref="A1:Q71" tableType="queryTable" totalsRowShown="0" headerRowDxfId="21" dataDxfId="19" headerRowBorderDxfId="20" tableBorderDxfId="18" totalsRowBorderDxfId="17">
   <autoFilter ref="A1:Q71" xr:uid="{D4DDD6FC-9AB0-4E27-B100-332C5258E37E}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:Q71">
     <sortCondition ref="A1:A71"/>
   </sortState>
   <tableColumns count="17">
-    <tableColumn id="1" xr3:uid="{08104193-2886-4FF4-8921-3158D7A7B5D5}" uniqueName="1" name="Run" queryTableFieldId="1" dataDxfId="18"/>
-    <tableColumn id="2" xr3:uid="{7C054C28-E3BC-4543-94CE-F53611EF06B7}" uniqueName="2" name="Bases" queryTableFieldId="2" dataDxfId="17"/>
-    <tableColumn id="3" xr3:uid="{ADF42818-3727-4002-82A9-12C0F87547B1}" uniqueName="3" name="BioProject" queryTableFieldId="3" dataDxfId="16"/>
-    <tableColumn id="4" xr3:uid="{78079789-B82A-44DB-B63A-3567B5F8BFFB}" uniqueName="4" name="BioSample" queryTableFieldId="4" dataDxfId="15"/>
-    <tableColumn id="5" xr3:uid="{8CC4EF86-1BF9-4C70-A455-239B6BA0E6C0}" uniqueName="5" name="Experiment" queryTableFieldId="5" dataDxfId="14"/>
-    <tableColumn id="6" xr3:uid="{7B82688F-5A73-4DE5-9EE5-2AC4BAEC71D4}" uniqueName="6" name="sample_name_incorrect" queryTableFieldId="6" dataDxfId="13"/>
-    <tableColumn id="7" xr3:uid="{13E76B27-CFDB-460A-94BA-D990D7126B99}" uniqueName="7" name="TF ID" queryTableFieldId="7" dataDxfId="12"/>
-    <tableColumn id="8" xr3:uid="{3AFC2BBC-8362-4C86-B60A-CC714D83C39E}" uniqueName="8" name="Sample ID" queryTableFieldId="8" dataDxfId="11"/>
-    <tableColumn id="9" xr3:uid="{D87ED850-B73B-47DC-8D38-FC93E72C9E29}" uniqueName="9" name="Cross" queryTableFieldId="9" dataDxfId="10"/>
-    <tableColumn id="10" xr3:uid="{60E986AE-2850-451A-83EA-FC9136093C20}" uniqueName="10" name="Family" queryTableFieldId="10" dataDxfId="9"/>
-    <tableColumn id="11" xr3:uid="{3BECC66F-C7FD-4A61-B85A-8AFD649B2FB0}" uniqueName="11" name="Sex" queryTableFieldId="11" dataDxfId="8"/>
-    <tableColumn id="16" xr3:uid="{4DE4FE7B-2921-4181-8540-496FC375EFB7}" uniqueName="16" name="Reciprocal Genotype" queryTableFieldId="18" dataDxfId="7"/>
-    <tableColumn id="18" xr3:uid="{2AE1460E-CE35-47C9-A107-BC4D77D67DDC}" uniqueName="18" name="Genotype" queryTableFieldId="20" dataDxfId="6"/>
-    <tableColumn id="17" xr3:uid="{10F931B8-E542-4DDB-9E3C-2B3E21E7EEC1}" uniqueName="17" name="Pairwise Cross" queryTableFieldId="19" dataDxfId="5"/>
-    <tableColumn id="13" xr3:uid="{DE2CE2BA-8696-4C1C-8A82-52220853E6A7}" uniqueName="13" name="original_fastq_name_R1" queryTableFieldId="14" dataDxfId="4"/>
-    <tableColumn id="14" xr3:uid="{DD7A34DD-98E1-41AE-9ED9-E9D738C46D29}" uniqueName="14" name="original_fastq_name_R2" queryTableFieldId="15" dataDxfId="3"/>
-    <tableColumn id="12" xr3:uid="{D586D41C-EF73-4229-A702-C14392310587}" uniqueName="12" name="Notes" queryTableFieldId="16" dataDxfId="2"/>
+    <tableColumn id="1" xr3:uid="{08104193-2886-4FF4-8921-3158D7A7B5D5}" uniqueName="1" name="Run" queryTableFieldId="1" dataDxfId="16"/>
+    <tableColumn id="2" xr3:uid="{7C054C28-E3BC-4543-94CE-F53611EF06B7}" uniqueName="2" name="Bases" queryTableFieldId="2" dataDxfId="15"/>
+    <tableColumn id="3" xr3:uid="{ADF42818-3727-4002-82A9-12C0F87547B1}" uniqueName="3" name="BioProject" queryTableFieldId="3" dataDxfId="14"/>
+    <tableColumn id="4" xr3:uid="{78079789-B82A-44DB-B63A-3567B5F8BFFB}" uniqueName="4" name="BioSample" queryTableFieldId="4" dataDxfId="13"/>
+    <tableColumn id="5" xr3:uid="{8CC4EF86-1BF9-4C70-A455-239B6BA0E6C0}" uniqueName="5" name="Experiment" queryTableFieldId="5" dataDxfId="12"/>
+    <tableColumn id="6" xr3:uid="{7B82688F-5A73-4DE5-9EE5-2AC4BAEC71D4}" uniqueName="6" name="sample_name_incorrect" queryTableFieldId="6" dataDxfId="11"/>
+    <tableColumn id="7" xr3:uid="{13E76B27-CFDB-460A-94BA-D990D7126B99}" uniqueName="7" name="TF ID" queryTableFieldId="7" dataDxfId="10"/>
+    <tableColumn id="8" xr3:uid="{3AFC2BBC-8362-4C86-B60A-CC714D83C39E}" uniqueName="8" name="Sample ID" queryTableFieldId="8" dataDxfId="9"/>
+    <tableColumn id="9" xr3:uid="{D87ED850-B73B-47DC-8D38-FC93E72C9E29}" uniqueName="9" name="Cross" queryTableFieldId="9" dataDxfId="8"/>
+    <tableColumn id="10" xr3:uid="{60E986AE-2850-451A-83EA-FC9136093C20}" uniqueName="10" name="Family" queryTableFieldId="10" dataDxfId="7"/>
+    <tableColumn id="11" xr3:uid="{3BECC66F-C7FD-4A61-B85A-8AFD649B2FB0}" uniqueName="11" name="Sex" queryTableFieldId="11" dataDxfId="6"/>
+    <tableColumn id="16" xr3:uid="{4DE4FE7B-2921-4181-8540-496FC375EFB7}" uniqueName="16" name="Reciprocal Genotype" queryTableFieldId="18" dataDxfId="5"/>
+    <tableColumn id="18" xr3:uid="{2AE1460E-CE35-47C9-A107-BC4D77D67DDC}" uniqueName="18" name="Genotype" queryTableFieldId="20" dataDxfId="4"/>
+    <tableColumn id="17" xr3:uid="{10F931B8-E542-4DDB-9E3C-2B3E21E7EEC1}" uniqueName="17" name="Pairwise Cross" queryTableFieldId="19" dataDxfId="3"/>
+    <tableColumn id="13" xr3:uid="{DE2CE2BA-8696-4C1C-8A82-52220853E6A7}" uniqueName="13" name="original_fastq_name_R1" queryTableFieldId="14" dataDxfId="2"/>
+    <tableColumn id="14" xr3:uid="{DD7A34DD-98E1-41AE-9ED9-E9D738C46D29}" uniqueName="14" name="original_fastq_name_R2" queryTableFieldId="15" dataDxfId="1"/>
+    <tableColumn id="12" xr3:uid="{D586D41C-EF73-4229-A702-C14392310587}" uniqueName="12" name="Notes" queryTableFieldId="16" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2821,7 +2825,7 @@
   <dimension ref="A1:Q71"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="12.21875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.21875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="12" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="11.88671875" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="15.77734375" bestFit="1" customWidth="1"/>
@@ -2854,7 +2858,7 @@
         <v>4</v>
       </c>
       <c r="F1" s="5" t="s">
-        <v>539</v>
+        <v>538</v>
       </c>
       <c r="G1" s="6" t="s">
         <v>280</v>
@@ -2872,13 +2876,13 @@
         <v>274</v>
       </c>
       <c r="L1" s="7" t="s">
+        <v>539</v>
+      </c>
+      <c r="M1" s="7" t="s">
         <v>540</v>
       </c>
-      <c r="M1" s="7" t="s">
+      <c r="N1" s="7" t="s">
         <v>541</v>
-      </c>
-      <c r="N1" s="7" t="s">
-        <v>542</v>
       </c>
       <c r="O1" s="5" t="s">
         <v>276</v>
@@ -2925,10 +2929,10 @@
         <v>283</v>
       </c>
       <c r="L2" s="13" t="s">
+        <v>544</v>
+      </c>
+      <c r="M2" s="13" t="s">
         <v>545</v>
-      </c>
-      <c r="M2" s="13" t="s">
-        <v>546</v>
       </c>
       <c r="N2" s="13">
         <v>1</v>
@@ -2976,10 +2980,10 @@
         <v>283</v>
       </c>
       <c r="L3" s="12" t="s">
+        <v>544</v>
+      </c>
+      <c r="M3" s="13" t="s">
         <v>545</v>
-      </c>
-      <c r="M3" s="13" t="s">
-        <v>546</v>
       </c>
       <c r="N3" s="12">
         <v>1</v>
@@ -3027,10 +3031,10 @@
         <v>283</v>
       </c>
       <c r="L4" s="12" t="s">
+        <v>544</v>
+      </c>
+      <c r="M4" s="13" t="s">
         <v>545</v>
-      </c>
-      <c r="M4" s="13" t="s">
-        <v>546</v>
       </c>
       <c r="N4" s="12">
         <v>1</v>
@@ -3078,10 +3082,10 @@
         <v>289</v>
       </c>
       <c r="L5" s="12" t="s">
-        <v>547</v>
+        <v>546</v>
       </c>
       <c r="M5" s="12" t="s">
-        <v>546</v>
+        <v>545</v>
       </c>
       <c r="N5" s="12">
         <v>1</v>
@@ -3129,10 +3133,10 @@
         <v>289</v>
       </c>
       <c r="L6" s="18" t="s">
-        <v>547</v>
+        <v>546</v>
       </c>
       <c r="M6" s="13" t="s">
-        <v>546</v>
+        <v>545</v>
       </c>
       <c r="N6" s="18">
         <v>1</v>
@@ -3180,10 +3184,10 @@
         <v>289</v>
       </c>
       <c r="L7" s="12" t="s">
-        <v>547</v>
+        <v>546</v>
       </c>
       <c r="M7" s="13" t="s">
-        <v>546</v>
+        <v>545</v>
       </c>
       <c r="N7" s="12">
         <v>1</v>
@@ -3231,10 +3235,10 @@
         <v>283</v>
       </c>
       <c r="L8" s="12" t="s">
-        <v>547</v>
+        <v>546</v>
       </c>
       <c r="M8" s="13" t="s">
-        <v>546</v>
+        <v>545</v>
       </c>
       <c r="N8" s="12">
         <v>1</v>
@@ -3282,10 +3286,10 @@
         <v>283</v>
       </c>
       <c r="L9" s="12" t="s">
-        <v>547</v>
+        <v>546</v>
       </c>
       <c r="M9" s="13" t="s">
-        <v>546</v>
+        <v>545</v>
       </c>
       <c r="N9" s="12">
         <v>1</v>
@@ -3333,10 +3337,10 @@
         <v>283</v>
       </c>
       <c r="L10" s="12" t="s">
-        <v>547</v>
+        <v>546</v>
       </c>
       <c r="M10" s="13" t="s">
-        <v>546</v>
+        <v>545</v>
       </c>
       <c r="N10" s="12">
         <v>1</v>
@@ -3347,8 +3351,8 @@
       <c r="P10" s="2" t="s">
         <v>522</v>
       </c>
-      <c r="Q10" s="16" t="s">
-        <v>523</v>
+      <c r="Q10" s="32" t="s">
+        <v>566</v>
       </c>
     </row>
     <row r="11" spans="1:17" x14ac:dyDescent="0.3">
@@ -3386,10 +3390,10 @@
         <v>289</v>
       </c>
       <c r="L11" s="19" t="s">
+        <v>547</v>
+      </c>
+      <c r="M11" s="19" t="s">
         <v>548</v>
-      </c>
-      <c r="M11" s="19" t="s">
-        <v>549</v>
       </c>
       <c r="N11" s="19">
         <v>1</v>
@@ -3437,10 +3441,10 @@
         <v>289</v>
       </c>
       <c r="L12" s="12" t="s">
+        <v>542</v>
+      </c>
+      <c r="M12" s="12" t="s">
         <v>543</v>
-      </c>
-      <c r="M12" s="12" t="s">
-        <v>544</v>
       </c>
       <c r="N12" s="12">
         <v>1</v>
@@ -3488,10 +3492,10 @@
         <v>289</v>
       </c>
       <c r="L13" s="12" t="s">
+        <v>547</v>
+      </c>
+      <c r="M13" s="19" t="s">
         <v>548</v>
-      </c>
-      <c r="M13" s="19" t="s">
-        <v>549</v>
       </c>
       <c r="N13" s="12">
         <v>1</v>
@@ -3539,10 +3543,10 @@
         <v>289</v>
       </c>
       <c r="L14" s="12" t="s">
+        <v>547</v>
+      </c>
+      <c r="M14" s="19" t="s">
         <v>548</v>
-      </c>
-      <c r="M14" s="19" t="s">
-        <v>549</v>
       </c>
       <c r="N14" s="12">
         <v>1</v>
@@ -3590,10 +3594,10 @@
         <v>283</v>
       </c>
       <c r="L15" s="19" t="s">
+        <v>547</v>
+      </c>
+      <c r="M15" s="19" t="s">
         <v>548</v>
-      </c>
-      <c r="M15" s="19" t="s">
-        <v>549</v>
       </c>
       <c r="N15" s="19">
         <v>1</v>
@@ -3641,10 +3645,10 @@
         <v>283</v>
       </c>
       <c r="L16" s="12" t="s">
+        <v>547</v>
+      </c>
+      <c r="M16" s="19" t="s">
         <v>548</v>
-      </c>
-      <c r="M16" s="19" t="s">
-        <v>549</v>
       </c>
       <c r="N16" s="12">
         <v>1</v>
@@ -3692,10 +3696,10 @@
         <v>283</v>
       </c>
       <c r="L17" s="12" t="s">
+        <v>547</v>
+      </c>
+      <c r="M17" s="19" t="s">
         <v>548</v>
-      </c>
-      <c r="M17" s="19" t="s">
-        <v>549</v>
       </c>
       <c r="N17" s="12">
         <v>1</v>
@@ -3743,10 +3747,10 @@
         <v>289</v>
       </c>
       <c r="L18" s="20" t="s">
+        <v>549</v>
+      </c>
+      <c r="M18" s="20" t="s">
         <v>550</v>
-      </c>
-      <c r="M18" s="20" t="s">
-        <v>551</v>
       </c>
       <c r="N18" s="20">
         <v>2</v>
@@ -3794,10 +3798,10 @@
         <v>289</v>
       </c>
       <c r="L19" s="20" t="s">
+        <v>549</v>
+      </c>
+      <c r="M19" s="20" t="s">
         <v>550</v>
-      </c>
-      <c r="M19" s="20" t="s">
-        <v>551</v>
       </c>
       <c r="N19" s="20">
         <v>2</v>
@@ -3845,10 +3849,10 @@
         <v>289</v>
       </c>
       <c r="L20" s="12" t="s">
+        <v>549</v>
+      </c>
+      <c r="M20" s="20" t="s">
         <v>550</v>
-      </c>
-      <c r="M20" s="20" t="s">
-        <v>551</v>
       </c>
       <c r="N20" s="12">
         <v>2</v>
@@ -3896,10 +3900,10 @@
         <v>283</v>
       </c>
       <c r="L21" s="20" t="s">
+        <v>549</v>
+      </c>
+      <c r="M21" s="20" t="s">
         <v>550</v>
-      </c>
-      <c r="M21" s="20" t="s">
-        <v>551</v>
       </c>
       <c r="N21" s="20">
         <v>2</v>
@@ -3947,10 +3951,10 @@
         <v>283</v>
       </c>
       <c r="L22" s="12" t="s">
+        <v>549</v>
+      </c>
+      <c r="M22" s="20" t="s">
         <v>550</v>
-      </c>
-      <c r="M22" s="20" t="s">
-        <v>551</v>
       </c>
       <c r="N22" s="12">
         <v>2</v>
@@ -3998,10 +4002,10 @@
         <v>289</v>
       </c>
       <c r="L23" s="12" t="s">
+        <v>542</v>
+      </c>
+      <c r="M23" s="12" t="s">
         <v>543</v>
-      </c>
-      <c r="M23" s="12" t="s">
-        <v>544</v>
       </c>
       <c r="N23" s="12">
         <v>1</v>
@@ -4049,10 +4053,10 @@
         <v>283</v>
       </c>
       <c r="L24" s="12" t="s">
+        <v>549</v>
+      </c>
+      <c r="M24" s="20" t="s">
         <v>550</v>
-      </c>
-      <c r="M24" s="20" t="s">
-        <v>551</v>
       </c>
       <c r="N24" s="12">
         <v>2</v>
@@ -4100,10 +4104,10 @@
         <v>289</v>
       </c>
       <c r="L25" s="12" t="s">
+        <v>551</v>
+      </c>
+      <c r="M25" s="12" t="s">
         <v>552</v>
-      </c>
-      <c r="M25" s="12" t="s">
-        <v>553</v>
       </c>
       <c r="N25" s="12">
         <v>2</v>
@@ -4151,10 +4155,10 @@
         <v>289</v>
       </c>
       <c r="L26" s="12" t="s">
+        <v>551</v>
+      </c>
+      <c r="M26" s="12" t="s">
         <v>552</v>
-      </c>
-      <c r="M26" s="12" t="s">
-        <v>553</v>
       </c>
       <c r="N26" s="12">
         <v>2</v>
@@ -4202,10 +4206,10 @@
         <v>289</v>
       </c>
       <c r="L27" s="12" t="s">
+        <v>551</v>
+      </c>
+      <c r="M27" s="12" t="s">
         <v>552</v>
-      </c>
-      <c r="M27" s="12" t="s">
-        <v>553</v>
       </c>
       <c r="N27" s="12">
         <v>2</v>
@@ -4253,10 +4257,10 @@
         <v>283</v>
       </c>
       <c r="L28" s="12" t="s">
+        <v>551</v>
+      </c>
+      <c r="M28" s="12" t="s">
         <v>552</v>
-      </c>
-      <c r="M28" s="12" t="s">
-        <v>553</v>
       </c>
       <c r="N28" s="12">
         <v>2</v>
@@ -4304,10 +4308,10 @@
         <v>283</v>
       </c>
       <c r="L29" s="12" t="s">
+        <v>551</v>
+      </c>
+      <c r="M29" s="12" t="s">
         <v>552</v>
-      </c>
-      <c r="M29" s="12" t="s">
-        <v>553</v>
       </c>
       <c r="N29" s="12">
         <v>2</v>
@@ -4355,10 +4359,10 @@
         <v>283</v>
       </c>
       <c r="L30" s="12" t="s">
+        <v>551</v>
+      </c>
+      <c r="M30" s="12" t="s">
         <v>552</v>
-      </c>
-      <c r="M30" s="12" t="s">
-        <v>553</v>
       </c>
       <c r="N30" s="12">
         <v>2</v>
@@ -4406,10 +4410,10 @@
         <v>289</v>
       </c>
       <c r="L31" s="12" t="s">
-        <v>554</v>
+        <v>553</v>
       </c>
       <c r="M31" s="12" t="s">
-        <v>553</v>
+        <v>552</v>
       </c>
       <c r="N31" s="12">
         <v>2</v>
@@ -4457,10 +4461,10 @@
         <v>289</v>
       </c>
       <c r="L32" s="12" t="s">
-        <v>554</v>
+        <v>553</v>
       </c>
       <c r="M32" s="12" t="s">
-        <v>553</v>
+        <v>552</v>
       </c>
       <c r="N32" s="12">
         <v>2</v>
@@ -4508,10 +4512,10 @@
         <v>289</v>
       </c>
       <c r="L33" s="12" t="s">
-        <v>554</v>
+        <v>553</v>
       </c>
       <c r="M33" s="12" t="s">
-        <v>553</v>
+        <v>552</v>
       </c>
       <c r="N33" s="12">
         <v>2</v>
@@ -4526,7 +4530,7 @@
     </row>
     <row r="34" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A34" s="9" t="s">
-        <v>524</v>
+        <v>523</v>
       </c>
       <c r="B34" s="10">
         <v>10153199532</v>
@@ -4535,16 +4539,16 @@
         <v>6</v>
       </c>
       <c r="D34" s="10" t="s">
+        <v>524</v>
+      </c>
+      <c r="E34" s="10" t="s">
         <v>525</v>
       </c>
-      <c r="E34" s="10" t="s">
+      <c r="F34" s="10" t="s">
         <v>526</v>
       </c>
-      <c r="F34" s="10" t="s">
+      <c r="G34" s="17" t="s">
         <v>527</v>
-      </c>
-      <c r="G34" s="17" t="s">
-        <v>528</v>
       </c>
       <c r="H34" s="12">
         <v>3</v>
@@ -4559,22 +4563,22 @@
         <v>289</v>
       </c>
       <c r="L34" s="12" t="s">
+        <v>542</v>
+      </c>
+      <c r="M34" s="12" t="s">
         <v>543</v>
-      </c>
-      <c r="M34" s="12" t="s">
-        <v>544</v>
       </c>
       <c r="N34" s="12">
         <v>1</v>
       </c>
       <c r="O34" s="15" t="s">
+        <v>528</v>
+      </c>
+      <c r="P34" s="15" t="s">
         <v>529</v>
       </c>
-      <c r="P34" s="15" t="s">
-        <v>530</v>
-      </c>
-      <c r="Q34" s="16" t="s">
-        <v>523</v>
+      <c r="Q34" s="32" t="s">
+        <v>567</v>
       </c>
     </row>
     <row r="35" spans="1:17" x14ac:dyDescent="0.3">
@@ -4612,10 +4616,10 @@
         <v>283</v>
       </c>
       <c r="L35" s="12" t="s">
-        <v>554</v>
+        <v>553</v>
       </c>
       <c r="M35" s="12" t="s">
-        <v>553</v>
+        <v>552</v>
       </c>
       <c r="N35" s="12">
         <v>2</v>
@@ -4663,10 +4667,10 @@
         <v>283</v>
       </c>
       <c r="L36" s="12" t="s">
-        <v>554</v>
+        <v>553</v>
       </c>
       <c r="M36" s="12" t="s">
-        <v>553</v>
+        <v>552</v>
       </c>
       <c r="N36" s="12">
         <v>2</v>
@@ -4714,10 +4718,10 @@
         <v>283</v>
       </c>
       <c r="L37" s="12" t="s">
-        <v>554</v>
+        <v>553</v>
       </c>
       <c r="M37" s="12" t="s">
-        <v>553</v>
+        <v>552</v>
       </c>
       <c r="N37" s="12">
         <v>2</v>
@@ -4765,10 +4769,10 @@
         <v>289</v>
       </c>
       <c r="L38" s="12" t="s">
+        <v>554</v>
+      </c>
+      <c r="M38" s="12" t="s">
         <v>555</v>
-      </c>
-      <c r="M38" s="12" t="s">
-        <v>556</v>
       </c>
       <c r="N38" s="12">
         <v>2</v>
@@ -4816,10 +4820,10 @@
         <v>283</v>
       </c>
       <c r="L39" s="12" t="s">
+        <v>554</v>
+      </c>
+      <c r="M39" s="12" t="s">
         <v>555</v>
-      </c>
-      <c r="M39" s="12" t="s">
-        <v>556</v>
       </c>
       <c r="N39" s="12">
         <v>2</v>
@@ -4830,8 +4834,8 @@
       <c r="P39" s="15" t="s">
         <v>410</v>
       </c>
-      <c r="Q39" s="16" t="s">
-        <v>557</v>
+      <c r="Q39" s="32" t="s">
+        <v>568</v>
       </c>
     </row>
     <row r="40" spans="1:17" x14ac:dyDescent="0.3">
@@ -4869,10 +4873,10 @@
         <v>289</v>
       </c>
       <c r="L40" s="12" t="s">
+        <v>554</v>
+      </c>
+      <c r="M40" s="12" t="s">
         <v>555</v>
-      </c>
-      <c r="M40" s="12" t="s">
-        <v>556</v>
       </c>
       <c r="N40" s="12">
         <v>2</v>
@@ -4920,10 +4924,10 @@
         <v>283</v>
       </c>
       <c r="L41" s="12" t="s">
+        <v>554</v>
+      </c>
+      <c r="M41" s="12" t="s">
         <v>555</v>
-      </c>
-      <c r="M41" s="12" t="s">
-        <v>556</v>
       </c>
       <c r="N41" s="12">
         <v>2</v>
@@ -4971,10 +4975,10 @@
         <v>283</v>
       </c>
       <c r="L42" s="12" t="s">
+        <v>554</v>
+      </c>
+      <c r="M42" s="12" t="s">
         <v>555</v>
-      </c>
-      <c r="M42" s="12" t="s">
-        <v>556</v>
       </c>
       <c r="N42" s="12">
         <v>2</v>
@@ -5022,10 +5026,10 @@
         <v>283</v>
       </c>
       <c r="L43" s="12" t="s">
+        <v>554</v>
+      </c>
+      <c r="M43" s="12" t="s">
         <v>555</v>
-      </c>
-      <c r="M43" s="12" t="s">
-        <v>556</v>
       </c>
       <c r="N43" s="12">
         <v>2</v>
@@ -5073,10 +5077,10 @@
         <v>289</v>
       </c>
       <c r="L44" s="12" t="s">
-        <v>558</v>
+        <v>556</v>
       </c>
       <c r="M44" s="12" t="s">
-        <v>559</v>
+        <v>557</v>
       </c>
       <c r="N44" s="12">
         <v>3</v>
@@ -5124,10 +5128,10 @@
         <v>283</v>
       </c>
       <c r="L45" s="12" t="s">
+        <v>542</v>
+      </c>
+      <c r="M45" s="12" t="s">
         <v>543</v>
-      </c>
-      <c r="M45" s="12" t="s">
-        <v>544</v>
       </c>
       <c r="N45" s="12">
         <v>1</v>
@@ -5175,10 +5179,10 @@
         <v>289</v>
       </c>
       <c r="L46" s="20" t="s">
-        <v>558</v>
+        <v>556</v>
       </c>
       <c r="M46" s="12" t="s">
-        <v>559</v>
+        <v>557</v>
       </c>
       <c r="N46" s="20">
         <v>3</v>
@@ -5226,10 +5230,10 @@
         <v>289</v>
       </c>
       <c r="L47" s="12" t="s">
-        <v>558</v>
+        <v>556</v>
       </c>
       <c r="M47" s="12" t="s">
-        <v>559</v>
+        <v>557</v>
       </c>
       <c r="N47" s="12">
         <v>3</v>
@@ -5277,10 +5281,10 @@
         <v>283</v>
       </c>
       <c r="L48" s="12" t="s">
-        <v>558</v>
+        <v>556</v>
       </c>
       <c r="M48" s="12" t="s">
-        <v>559</v>
+        <v>557</v>
       </c>
       <c r="N48" s="12">
         <v>3</v>
@@ -5328,10 +5332,10 @@
         <v>283</v>
       </c>
       <c r="L49" s="12" t="s">
-        <v>558</v>
+        <v>556</v>
       </c>
       <c r="M49" s="12" t="s">
-        <v>559</v>
+        <v>557</v>
       </c>
       <c r="N49" s="12">
         <v>3</v>
@@ -5379,10 +5383,10 @@
         <v>283</v>
       </c>
       <c r="L50" s="12" t="s">
-        <v>558</v>
+        <v>556</v>
       </c>
       <c r="M50" s="12" t="s">
-        <v>559</v>
+        <v>557</v>
       </c>
       <c r="N50" s="12">
         <v>3</v>
@@ -5430,10 +5434,10 @@
         <v>289</v>
       </c>
       <c r="L51" s="12" t="s">
-        <v>560</v>
+        <v>558</v>
       </c>
       <c r="M51" s="12" t="s">
-        <v>561</v>
+        <v>559</v>
       </c>
       <c r="N51" s="12">
         <v>3</v>
@@ -5481,10 +5485,10 @@
         <v>289</v>
       </c>
       <c r="L52" s="12" t="s">
-        <v>560</v>
+        <v>558</v>
       </c>
       <c r="M52" s="12" t="s">
-        <v>561</v>
+        <v>559</v>
       </c>
       <c r="N52" s="12">
         <v>3</v>
@@ -5532,10 +5536,10 @@
         <v>283</v>
       </c>
       <c r="L53" s="21" t="s">
-        <v>560</v>
+        <v>558</v>
       </c>
       <c r="M53" s="12" t="s">
-        <v>561</v>
+        <v>559</v>
       </c>
       <c r="N53" s="21">
         <v>3</v>
@@ -5583,10 +5587,10 @@
         <v>283</v>
       </c>
       <c r="L54" s="12" t="s">
-        <v>560</v>
+        <v>558</v>
       </c>
       <c r="M54" s="12" t="s">
-        <v>561</v>
+        <v>559</v>
       </c>
       <c r="N54" s="12">
         <v>3</v>
@@ -5634,10 +5638,10 @@
         <v>283</v>
       </c>
       <c r="L55" s="12" t="s">
+        <v>542</v>
+      </c>
+      <c r="M55" s="12" t="s">
         <v>543</v>
-      </c>
-      <c r="M55" s="12" t="s">
-        <v>544</v>
       </c>
       <c r="N55" s="12">
         <v>1</v>
@@ -5685,10 +5689,10 @@
         <v>283</v>
       </c>
       <c r="L56" s="12" t="s">
-        <v>560</v>
+        <v>558</v>
       </c>
       <c r="M56" s="12" t="s">
-        <v>561</v>
+        <v>559</v>
       </c>
       <c r="N56" s="12">
         <v>3</v>
@@ -5736,10 +5740,10 @@
         <v>289</v>
       </c>
       <c r="L57" s="12" t="s">
-        <v>562</v>
+        <v>560</v>
       </c>
       <c r="M57" s="12" t="s">
-        <v>561</v>
+        <v>559</v>
       </c>
       <c r="N57" s="12">
         <v>3</v>
@@ -5787,10 +5791,10 @@
         <v>289</v>
       </c>
       <c r="L58" s="12" t="s">
-        <v>562</v>
+        <v>560</v>
       </c>
       <c r="M58" s="12" t="s">
-        <v>561</v>
+        <v>559</v>
       </c>
       <c r="N58" s="12">
         <v>3</v>
@@ -5838,10 +5842,10 @@
         <v>283</v>
       </c>
       <c r="L59" s="12" t="s">
-        <v>562</v>
+        <v>560</v>
       </c>
       <c r="M59" s="12" t="s">
-        <v>561</v>
+        <v>559</v>
       </c>
       <c r="N59" s="12">
         <v>3</v>
@@ -5889,10 +5893,10 @@
         <v>283</v>
       </c>
       <c r="L60" s="12" t="s">
-        <v>562</v>
+        <v>560</v>
       </c>
       <c r="M60" s="12" t="s">
-        <v>561</v>
+        <v>559</v>
       </c>
       <c r="N60" s="12">
         <v>3</v>
@@ -5940,10 +5944,10 @@
         <v>283</v>
       </c>
       <c r="L61" s="12" t="s">
-        <v>562</v>
+        <v>560</v>
       </c>
       <c r="M61" s="12" t="s">
-        <v>561</v>
+        <v>559</v>
       </c>
       <c r="N61" s="12">
         <v>3</v>
@@ -5991,10 +5995,10 @@
         <v>289</v>
       </c>
       <c r="L62" s="19" t="s">
-        <v>563</v>
+        <v>561</v>
       </c>
       <c r="M62" s="19" t="s">
-        <v>564</v>
+        <v>562</v>
       </c>
       <c r="N62" s="19">
         <v>3</v>
@@ -6042,10 +6046,10 @@
         <v>289</v>
       </c>
       <c r="L63" s="12" t="s">
-        <v>563</v>
+        <v>561</v>
       </c>
       <c r="M63" s="19" t="s">
-        <v>564</v>
+        <v>562</v>
       </c>
       <c r="N63" s="12">
         <v>3</v>
@@ -6060,7 +6064,7 @@
     </row>
     <row r="64" spans="1:17" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A64" s="9" t="s">
-        <v>531</v>
+        <v>530</v>
       </c>
       <c r="B64" s="10">
         <v>16388897646</v>
@@ -6069,19 +6073,19 @@
         <v>6</v>
       </c>
       <c r="D64" s="10" t="s">
+        <v>531</v>
+      </c>
+      <c r="E64" s="10" t="s">
         <v>532</v>
       </c>
-      <c r="E64" s="10" t="s">
+      <c r="F64" s="10" t="s">
         <v>533</v>
       </c>
-      <c r="F64" s="10" t="s">
+      <c r="G64" s="11" t="s">
         <v>534</v>
       </c>
-      <c r="G64" s="11" t="s">
+      <c r="H64" s="12" t="s">
         <v>535</v>
-      </c>
-      <c r="H64" s="12" t="s">
-        <v>536</v>
       </c>
       <c r="I64" s="19" t="s">
         <v>489</v>
@@ -6093,22 +6097,22 @@
         <v>289</v>
       </c>
       <c r="L64" s="19" t="s">
-        <v>563</v>
+        <v>561</v>
       </c>
       <c r="M64" s="19" t="s">
-        <v>564</v>
+        <v>562</v>
       </c>
       <c r="N64" s="19">
         <v>3</v>
       </c>
       <c r="O64" s="15" t="s">
+        <v>536</v>
+      </c>
+      <c r="P64" s="15" t="s">
         <v>537</v>
       </c>
-      <c r="P64" s="15" t="s">
-        <v>538</v>
-      </c>
-      <c r="Q64" s="16" t="s">
-        <v>523</v>
+      <c r="Q64" s="32" t="s">
+        <v>567</v>
       </c>
     </row>
     <row r="65" spans="1:17" x14ac:dyDescent="0.3">
@@ -6146,10 +6150,10 @@
         <v>283</v>
       </c>
       <c r="L65" s="12" t="s">
+        <v>542</v>
+      </c>
+      <c r="M65" s="12" t="s">
         <v>543</v>
-      </c>
-      <c r="M65" s="12" t="s">
-        <v>544</v>
       </c>
       <c r="N65" s="12">
         <v>1</v>
@@ -6197,10 +6201,10 @@
         <v>283</v>
       </c>
       <c r="L66" s="12" t="s">
-        <v>563</v>
+        <v>561</v>
       </c>
       <c r="M66" s="19" t="s">
-        <v>564</v>
+        <v>562</v>
       </c>
       <c r="N66" s="12">
         <v>3</v>
@@ -6212,7 +6216,7 @@
         <v>497</v>
       </c>
       <c r="Q66" s="16" t="s">
-        <v>565</v>
+        <v>563</v>
       </c>
     </row>
     <row r="67" spans="1:17" x14ac:dyDescent="0.3">
@@ -6250,10 +6254,10 @@
         <v>283</v>
       </c>
       <c r="L67" s="25" t="s">
-        <v>563</v>
+        <v>561</v>
       </c>
       <c r="M67" s="19" t="s">
-        <v>564</v>
+        <v>562</v>
       </c>
       <c r="N67" s="25">
         <v>3</v>
@@ -6265,7 +6269,7 @@
         <v>500</v>
       </c>
       <c r="Q67" s="27" t="s">
-        <v>566</v>
+        <v>564</v>
       </c>
     </row>
     <row r="68" spans="1:17" x14ac:dyDescent="0.3">
@@ -6303,10 +6307,10 @@
         <v>283</v>
       </c>
       <c r="L68" s="12" t="s">
-        <v>563</v>
+        <v>561</v>
       </c>
       <c r="M68" s="19" t="s">
-        <v>564</v>
+        <v>562</v>
       </c>
       <c r="N68" s="12">
         <v>3</v>
@@ -6318,7 +6322,7 @@
         <v>503</v>
       </c>
       <c r="Q68" s="10" t="s">
-        <v>567</v>
+        <v>565</v>
       </c>
     </row>
     <row r="69" spans="1:17" x14ac:dyDescent="0.3">
@@ -6356,10 +6360,10 @@
         <v>289</v>
       </c>
       <c r="L69" s="29" t="s">
+        <v>544</v>
+      </c>
+      <c r="M69" s="13" t="s">
         <v>545</v>
-      </c>
-      <c r="M69" s="13" t="s">
-        <v>546</v>
       </c>
       <c r="N69" s="29">
         <v>1</v>
@@ -6407,10 +6411,10 @@
         <v>289</v>
       </c>
       <c r="L70" s="12" t="s">
+        <v>544</v>
+      </c>
+      <c r="M70" s="13" t="s">
         <v>545</v>
-      </c>
-      <c r="M70" s="13" t="s">
-        <v>546</v>
       </c>
       <c r="N70" s="12">
         <v>1</v>
@@ -6458,10 +6462,10 @@
         <v>289</v>
       </c>
       <c r="L71" s="31" t="s">
+        <v>544</v>
+      </c>
+      <c r="M71" s="13" t="s">
         <v>545</v>
-      </c>
-      <c r="M71" s="13" t="s">
-        <v>546</v>
       </c>
       <c r="N71" s="31">
         <v>1</v>

</xml_diff>